<commit_message>
test(calculators): added note about pending feedback to the formula in the test sheet
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/6.2-pasture-residues.xlsx
+++ b/packages/calculators/src/modules/test/6.2-pasture-residues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4C285A5-52F6-CE45-A817-500075BA5C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB2E7BA-DCAD-274A-9855-2AB25038F3AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15940" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
+    <workbookView xWindow="-20" yWindow="620" windowWidth="28800" windowHeight="15900" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
   <sheets>
     <sheet name="6.2.1.1" sheetId="1" r:id="rId1"/>
@@ -166,6 +166,69 @@
     </r>
   </si>
   <si>
+    <t>En2o</t>
+  </si>
+  <si>
+    <t>Mp</t>
+  </si>
+  <si>
+    <t>Ap</t>
+  </si>
+  <si>
+    <t>Yp</t>
+  </si>
+  <si>
+    <t>FFODp</t>
+  </si>
+  <si>
+    <t>Fraction of pasture removed</t>
+  </si>
+  <si>
+    <t>Table A.2.1.3</t>
+  </si>
+  <si>
+    <t>Rbgp</t>
+  </si>
+  <si>
+    <t>Ncagp</t>
+  </si>
+  <si>
+    <t>NCbgp</t>
+  </si>
+  <si>
+    <t>RBGp</t>
+  </si>
+  <si>
+    <t>NCBGp</t>
+  </si>
+  <si>
+    <t>Pasture type</t>
+  </si>
+  <si>
+    <t>Annual grass</t>
+  </si>
+  <si>
+    <t>Grass clover mixture</t>
+  </si>
+  <si>
+    <t>Lucerne</t>
+  </si>
+  <si>
+    <t>Other legume</t>
+  </si>
+  <si>
+    <t>Perennial pasture</t>
+  </si>
+  <si>
+    <t>Method 2</t>
+  </si>
+  <si>
+    <t>Average yield per hectare in t</t>
+  </si>
+  <si>
+    <t>Area of pasture in hectares</t>
+  </si>
+  <si>
     <r>
       <t>𝑀</t>
     </r>
@@ -221,7 +284,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t>× 10</t>
+      <t>× 10^</t>
     </r>
     <r>
       <rPr>
@@ -230,7 +293,7 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t>−3</t>
+      <t>3</t>
     </r>
     <r>
       <rPr>
@@ -275,74 +338,11 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t>) + (𝐴𝑝 × (𝑌 𝑝 × 10−3) × 𝑅𝐵𝐺𝑝 × 𝑁𝐶𝐵𝐺𝑝)</t>
-    </r>
-  </si>
-  <si>
-    <t>En2o</t>
-  </si>
-  <si>
-    <t>Mp</t>
-  </si>
-  <si>
-    <t>Ap</t>
-  </si>
-  <si>
-    <t>Yp</t>
-  </si>
-  <si>
-    <t>FFODp</t>
-  </si>
-  <si>
-    <t>Fraction of pasture removed</t>
-  </si>
-  <si>
-    <t>Table A.2.1.3</t>
-  </si>
-  <si>
-    <t>Rbgp</t>
-  </si>
-  <si>
-    <t>Ncagp</t>
-  </si>
-  <si>
-    <t>NCbgp</t>
-  </si>
-  <si>
-    <t>RBGp</t>
-  </si>
-  <si>
-    <t>NCBGp</t>
-  </si>
-  <si>
-    <t>Pasture type</t>
-  </si>
-  <si>
-    <t>Annual grass</t>
-  </si>
-  <si>
-    <t>Grass clover mixture</t>
-  </si>
-  <si>
-    <t>Lucerne</t>
-  </si>
-  <si>
-    <t>Other legume</t>
-  </si>
-  <si>
-    <t>Perennial pasture</t>
-  </si>
-  <si>
-    <t>Method 2</t>
-  </si>
-  <si>
-    <t>Average yield per hectare in t</t>
-  </si>
-  <si>
-    <t>Area of pasture in hectares</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOTE: Pending feedback, I think this formula is incorrect. Multiplying by 10^-3 converts the yield in tonnes to gigagrams, not kilograms. I've implemented the </t>
+      <t>) + (𝐴𝑝 × (𝑌 𝑝 × 10^3) × 𝑅𝐵𝐺𝑝 × 𝑁𝐶𝐵𝐺𝑝)</t>
+    </r>
+  </si>
+  <si>
+    <t>NOTE: Pending feedback, I think this formula is incorrect. Multiplying by 10^-3 converts the yield in tonnes to gigagrams, not kilograms. I've implemented this with what I think is the correct conversion</t>
   </si>
 </sst>
 </file>
@@ -815,20 +815,20 @@
     </row>
     <row r="3" spans="1:16" ht="34">
       <c r="C3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
       <c r="J3" s="1" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L3" s="1"/>
     </row>
@@ -837,34 +837,34 @@
         <v>9</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
         <v>23</v>
       </c>
-      <c r="H4" t="s">
-        <v>24</v>
-      </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K4" t="s">
         <v>3</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N4" s="6" t="s">
         <v>1</v>
@@ -875,7 +875,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5">
         <v>5000</v>
@@ -919,7 +919,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6">
         <v>50</v>
@@ -963,7 +963,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7">
         <v>600</v>
@@ -1007,7 +1007,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8">
         <v>7000</v>
@@ -1053,7 +1053,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9">
         <v>50</v>
@@ -1099,7 +1099,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10">
         <v>50</v>
@@ -1304,7 +1304,7 @@
     </row>
     <row r="15" spans="1:16">
       <c r="B15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15" s="12" t="str">
         <f t="shared" si="8"/>
@@ -1388,7 +1388,7 @@
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C17">
         <v>50</v>
@@ -1431,7 +1431,7 @@
         <v>7</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C18">
         <v>600</v>
@@ -1476,7 +1476,7 @@
         <v>8</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C19">
         <v>7000</v>
@@ -1514,22 +1514,22 @@
         <v>7.1499999999999986</v>
       </c>
       <c r="N19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O19" s="2" t="s">
+      <c r="Q19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="S19" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="P19" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="R19" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="S19" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:22">
@@ -1537,7 +1537,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C20">
         <v>50</v>
@@ -1575,7 +1575,7 @@
         <v>8.3678571428571435E-2</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O20" s="2">
         <v>4.41</v>
@@ -1595,7 +1595,7 @@
     </row>
     <row r="21" spans="1:22">
       <c r="N21" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O21" s="2">
         <v>8.34</v>
@@ -1615,7 +1615,7 @@
     </row>
     <row r="22" spans="1:22">
       <c r="N22" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O22" s="2">
         <v>8.6199999999999992</v>
@@ -1639,7 +1639,7 @@
     <row r="23" spans="1:22">
       <c r="B23" s="2"/>
       <c r="N23" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O23" s="2">
         <v>5.62</v>
@@ -1663,7 +1663,7 @@
     <row r="24" spans="1:22">
       <c r="B24" s="2"/>
       <c r="N24" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O24" s="2">
         <v>8.35</v>

</xml_diff>